<commit_message>
Add full mobile responsiveness, PWA support, WhatsApp sharing
- Collapsible sidebar with hamburger menu on mobile (<768px)
- Responsive grids, tables, forms, dialogs across all 25+ components
- Hide less important table columns on small screens
- PWA manifest, service worker, app icons for installability
- WhatsApp share dialog for analytics reports
- SVG favicon, updated index.html with Apple meta tags

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/farm-tracker/scripts/Details.xlsx
+++ b/farm-tracker/scripts/Details.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="70">
   <si>
     <t>Date</t>
   </si>
@@ -134,9 +134,6 @@
     <t>6*850=5,100 labour saturday</t>
   </si>
   <si>
-    <t>Inventry</t>
-  </si>
-  <si>
     <t xml:space="preserve">kairu </t>
   </si>
   <si>
@@ -155,15 +152,34 @@
     <t>Chicks</t>
   </si>
   <si>
-    <t>70 chicks -- 30 karpu ,40 sonaly,  total = 10700</t>
+    <t>animal stock</t>
   </si>
   <si>
-    <t>mannur clean</t>
+    <t>70 chicks -- 30 karpu ,40 sonaly,  total = 10700</t>
   </si>
   <si>
     <t>3 load earuvu 3*1500=4,500 
 Old 2 load earuvu 2*1500=3,000 
 Total ₹=7500</t>
+  </si>
+  <si>
+    <t>11*400=4,400   for plant tie</t>
+  </si>
+  <si>
+    <t>493  for kairu</t>
+  </si>
+  <si>
+    <t>Animal Stock</t>
+  </si>
+  <si>
+    <t>120*83=9,960 
+Petrol =1200
+1200+9960=11,160    , food 1420</t>
+  </si>
+  <si>
+    <t xml:space="preserve">120*83=9,960 
+Petrol =1200
+1200+9960=11,160    </t>
   </si>
   <si>
     <t>Income Source</t>
@@ -386,11 +402,11 @@
             </c:numRef>
           </c:val>
         </c:ser>
-        <c:axId val="1950712538"/>
-        <c:axId val="1113267654"/>
+        <c:axId val="437656224"/>
+        <c:axId val="1020360200"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="1950712538"/>
+        <c:axId val="437656224"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -442,10 +458,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1113267654"/>
+        <c:crossAx val="1020360200"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1113267654"/>
+        <c:axId val="1020360200"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -520,7 +536,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1950712538"/>
+        <c:crossAx val="437656224"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -1178,10 +1194,10 @@
         <v>16</v>
       </c>
       <c r="C17" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="D17" s="7" t="s">
         <v>36</v>
-      </c>
-      <c r="D17" s="7" t="s">
-        <v>37</v>
       </c>
       <c r="E17" s="6">
         <v>660.0</v>
@@ -1204,7 +1220,7 @@
         <v>23</v>
       </c>
       <c r="D18" s="7" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E18" s="6">
         <v>2000.0</v>
@@ -1310,7 +1326,7 @@
         <v>17</v>
       </c>
       <c r="D23" s="7" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E23" s="6">
         <v>1382.0</v>
@@ -1333,7 +1349,7 @@
         <v>17</v>
       </c>
       <c r="D24" s="7" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E24" s="6">
         <v>1550.0</v>
@@ -1350,10 +1366,10 @@
         <v>46144.0</v>
       </c>
       <c r="B25" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="C25" s="7" t="s">
         <v>41</v>
-      </c>
-      <c r="C25" s="5" t="s">
-        <v>36</v>
       </c>
       <c r="D25" s="7" t="s">
         <v>42</v>
@@ -1373,10 +1389,10 @@
         <v>46144.0</v>
       </c>
       <c r="B26" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="C26" s="5" t="s">
         <v>41</v>
-      </c>
-      <c r="C26" s="5" t="s">
-        <v>36</v>
       </c>
       <c r="D26" s="7" t="s">
         <v>42</v>
@@ -1399,10 +1415,10 @@
         <v>16</v>
       </c>
       <c r="C27" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="D27" s="7" t="s">
         <v>43</v>
-      </c>
-      <c r="D27" s="7" t="s">
-        <v>44</v>
       </c>
       <c r="E27" s="6">
         <v>7500.0</v>
@@ -1415,36 +1431,96 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="10"/>
-      <c r="B28" s="11"/>
-      <c r="C28" s="11"/>
-      <c r="E28" s="12"/>
-      <c r="F28" s="11"/>
-      <c r="G28" s="11"/>
+      <c r="A28" s="8">
+        <v>46160.0</v>
+      </c>
+      <c r="B28" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C28" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="D28" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="E28" s="6">
+        <v>4400.0</v>
+      </c>
+      <c r="F28" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="G28" s="5" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="29">
-      <c r="A29" s="10"/>
-      <c r="B29" s="11"/>
-      <c r="C29" s="11"/>
-      <c r="E29" s="12"/>
-      <c r="F29" s="11"/>
-      <c r="G29" s="11"/>
+      <c r="A29" s="8">
+        <v>46160.0</v>
+      </c>
+      <c r="B29" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C29" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="D29" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="E29" s="6">
+        <v>493.0</v>
+      </c>
+      <c r="F29" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="G29" s="5" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="30">
-      <c r="A30" s="10"/>
-      <c r="B30" s="11"/>
-      <c r="C30" s="11"/>
-      <c r="E30" s="12"/>
-      <c r="F30" s="11"/>
-      <c r="G30" s="11"/>
+      <c r="A30" s="8">
+        <v>46175.0</v>
+      </c>
+      <c r="B30" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="C30" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="D30" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="E30" s="6">
+        <v>7000.0</v>
+      </c>
+      <c r="F30" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="G30" s="5" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="31">
-      <c r="A31" s="10"/>
-      <c r="B31" s="11"/>
-      <c r="C31" s="11"/>
-      <c r="E31" s="12"/>
-      <c r="F31" s="11"/>
-      <c r="G31" s="11"/>
+      <c r="A31" s="8">
+        <v>46175.0</v>
+      </c>
+      <c r="B31" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="C31" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="D31" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="E31" s="6">
+        <v>4160.0</v>
+      </c>
+      <c r="F31" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="G31" s="5" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="10"/>
@@ -2003,20 +2079,23 @@
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="F2:F100">
       <formula1>"KK,SK,Bank,Gold Loan"</formula1>
     </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="C3:C24 C26:C100">
+      <formula1>"Maintenance,Animal Stock,People,Travel,Food,Loan Repaymnet,mannur clean,animal stock"</formula1>
+    </dataValidation>
     <dataValidation type="custom" allowBlank="1" showDropDown="1" showErrorMessage="1" sqref="A2:A100">
       <formula1>OR(NOT(ISERROR(DATEVALUE(A2))), AND(ISNUMBER(A2), LEFT(CELL("format", A2))="D"))</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="C2">
-      <formula1>"Inventry,Loan Repayment,People,Travel,Food"</formula1>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="C25">
+      <formula1>"Inventry,animal stock"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="B2:B100">
       <formula1>"Goat,Dragon,Chicks"</formula1>
     </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="C2">
+      <formula1>"Inventry,Loan Repayment,People,Travel,Food,Farm Equipment,Animal Stock"</formula1>
+    </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="G2:G100">
       <formula1>"UPI,CASH"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="C3:C100">
-      <formula1>"Maintenance,Inventry,People,Travel,Food,Loan Repaymnet,mannur clean"</formula1>
     </dataValidation>
   </dataValidations>
   <drawing r:id="rId1"/>
@@ -2713,7 +2792,7 @@
         <v>1</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>3</v>
@@ -2722,7 +2801,7 @@
         <v>4</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="G1" s="2" t="s">
         <v>6</v>
@@ -7754,15 +7833,15 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="B2" s="13">
         <f>SUMIFS(Expenses!E:E,Expenses!B:B,"Goat")</f>
@@ -7771,16 +7850,16 @@
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="B3" s="13">
         <f>SUMIFS(Expenses!E:E,Expenses!B:B,"Dragon")</f>
-        <v>46392</v>
+        <v>51285</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="B4" s="13">
         <f>SUM(Income!E:E)</f>
@@ -7789,38 +7868,38 @@
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="B5" s="13">
         <f>SUM(Expenses!E:E)</f>
-        <v>299690</v>
+        <v>315743</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="B6" s="13">
         <f>SUMIFS(Expenses!E:E,Expenses!F:F,"KK")</f>
-        <v>197718</v>
+        <v>204718</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="B7" s="13">
         <f>SUMIFS(Expenses!E:E,Expenses!F:F,"SK")</f>
-        <v>53212</v>
+        <v>62265</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="B8" s="13">
         <f>B4-B5</f>
-        <v>-299690</v>
+        <v>-315743</v>
       </c>
     </row>
   </sheetData>
@@ -7850,7 +7929,7 @@
         <v>182353.0</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
     </row>
     <row r="3">
@@ -7863,7 +7942,7 @@
     </row>
     <row r="4">
       <c r="B4" s="7" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="C4" s="7">
         <v>61000.0</v>
@@ -7871,36 +7950,36 @@
     </row>
     <row r="6">
       <c r="A6" s="7" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="14" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="C7" s="14">
         <v>120000.0</v>
       </c>
       <c r="D7" s="14" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="E7" s="14" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="F7" s="14" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="G7" s="14" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="H7" s="15"/>
       <c r="I7" s="15"/>

</xml_diff>